<commit_message>
IDMA preparing for re-exam
</commit_message>
<xml_diff>
--- a/ExamOral_2026/RegistrationList_OralRe-exam_IDMA26_NDAB23K02E.xlsx
+++ b/ExamOral_2026/RegistrationList_OralRe-exam_IDMA26_NDAB23K02E.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\Teaching\IDMA26\ExamOral_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17AE7078-A408-4D20-AA7F-25FC69F71218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF862A54-9FAD-4BE4-AB63-4B15B72C7338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7E1502AD-AEB5-4B5A-AE21-DE13E93375EA}"/>
+    <workbookView xWindow="1509" yWindow="1509" windowWidth="19337" windowHeight="9120" xr2:uid="{A5F70A67-53ED-464E-B5A6-15044B1BDE27}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <t>ADM</t>
   </si>
@@ -62,10 +62,13 @@
     <t>STUD_ID</t>
   </si>
   <si>
+    <t>STUD_NAVN</t>
+  </si>
+  <si>
     <t>TILM_STATUS</t>
   </si>
   <si>
-    <t>5100 Datalogisk Institut samt underordnede enheder</t>
+    <t>Alle</t>
   </si>
   <si>
     <t>Termin         : Eksamen blok 3 2025-2026, reeksamen</t>
@@ -83,46 +86,28 @@
     <t>Introduktion til diskret matematik og algoritmer</t>
   </si>
   <si>
-    <t>HMF512</t>
+    <t>VJZ343</t>
+  </si>
+  <si>
+    <t>Møller, Siw Foged</t>
   </si>
   <si>
     <t>tilmeldt</t>
   </si>
   <si>
-    <t>LWH753</t>
-  </si>
-  <si>
-    <t>DQR746</t>
-  </si>
-  <si>
-    <t>ZBT570</t>
-  </si>
-  <si>
-    <t>ZJM580</t>
-  </si>
-  <si>
-    <t>VJZ343</t>
-  </si>
-  <si>
     <t>TZQ775</t>
   </si>
   <si>
-    <t>LDS147</t>
-  </si>
-  <si>
-    <t>GRL379</t>
+    <t>Skovborg, Noah Gyldenløve</t>
   </si>
   <si>
     <t>Kolonne1</t>
   </si>
   <si>
-    <t>Kolonne2</t>
-  </si>
-  <si>
     <t>MF (Skriv MF hvis MF, ellers blank)</t>
   </si>
   <si>
-    <t>OK</t>
+    <t xml:space="preserve">   OK, but listed on both registration lists!?</t>
   </si>
 </sst>
 </file>
@@ -191,20 +176,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9D75EA38-54AB-488A-8E0A-9C9DE7F49A8A}" name="Tabel1" displayName="Tabel1" ref="A1:K10" totalsRowShown="0">
-  <autoFilter ref="A1:K10" xr:uid="{9D75EA38-54AB-488A-8E0A-9C9DE7F49A8A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A3C70D-94A5-4427-B242-2B5E82D3D199}" name="Tabel1" displayName="Tabel1" ref="A1:K3" totalsRowShown="0">
+  <autoFilter ref="A1:K3" xr:uid="{61A3C70D-94A5-4427-B242-2B5E82D3D199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{6D5B5893-B6D3-474B-A356-7D55B34E5293}" name="ADM"/>
-    <tableColumn id="2" xr3:uid="{D863E338-35EB-4116-B255-F07A88D193D3}" name="TERMIN"/>
-    <tableColumn id="3" xr3:uid="{1AB0D960-885F-4976-81FA-36D253E2FB4C}" name="EKSAMENSTYPE"/>
-    <tableColumn id="4" xr3:uid="{9F244463-10E0-487C-9DD5-D9C9D9246B96}" name="EKS_AKT_KODE"/>
-    <tableColumn id="5" xr3:uid="{7E82DB3B-7926-4D80-87C9-F5DD6DD946F6}" name="VALG"/>
-    <tableColumn id="6" xr3:uid="{F5FFB148-C36F-4D63-B353-E9D4A4125465}" name="EKS_AKT_NAVN"/>
-    <tableColumn id="7" xr3:uid="{45BE70A6-C764-4B62-BC3F-E6EC3086C6B4}" name="STUD_ID"/>
-    <tableColumn id="8" xr3:uid="{E8CDD589-174F-4B6D-AB61-F0D186E9DB06}" name="TILM_STATUS"/>
-    <tableColumn id="9" xr3:uid="{9236E026-5787-4C16-9933-83F2D801B654}" name="Kolonne1"/>
-    <tableColumn id="10" xr3:uid="{29455400-9ADB-4051-8EA5-D74EE6AB3347}" name="Kolonne2"/>
-    <tableColumn id="11" xr3:uid="{8ADECD65-9638-41D7-999A-0D50300C170C}" name="MF (Skriv MF hvis MF, ellers blank)" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{F24EE80C-A3AD-481A-847D-CB70049D4622}" name="ADM"/>
+    <tableColumn id="2" xr3:uid="{7A42CEEC-3EB6-426D-8220-9B58DC8DC681}" name="TERMIN"/>
+    <tableColumn id="3" xr3:uid="{2C68D63D-CE47-4DB2-A0E5-F67D420C18B6}" name="EKSAMENSTYPE"/>
+    <tableColumn id="4" xr3:uid="{9CD70A4A-ADF7-430F-A2A3-37C065612DF7}" name="EKS_AKT_KODE"/>
+    <tableColumn id="5" xr3:uid="{D3292058-5D6C-4C9F-8F0D-CB7D9C212C4B}" name="VALG"/>
+    <tableColumn id="6" xr3:uid="{4B062CA1-A232-40C0-8EDC-BE3C889F6820}" name="EKS_AKT_NAVN"/>
+    <tableColumn id="7" xr3:uid="{94283505-DE09-4D3C-A9CA-A01EA71F8C30}" name="STUD_ID"/>
+    <tableColumn id="8" xr3:uid="{134890EE-89D2-4107-99B3-832D52882C90}" name="STUD_NAVN"/>
+    <tableColumn id="9" xr3:uid="{D4010A9E-5F86-4C77-A0A0-C880D84BFA37}" name="TILM_STATUS"/>
+    <tableColumn id="10" xr3:uid="{E70BEECB-0BFC-4118-9605-E4EFEFEAC352}" name="Kolonne1"/>
+    <tableColumn id="11" xr3:uid="{F37E72D8-7BA1-4DFB-94D2-A94C60B48F47}" name="MF (Skriv MF hvis MF, ellers blank)" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -526,19 +511,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DCCF5A3-B872-4E23-9E71-334503FCF467}">
-  <dimension ref="A1:K10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B09B5899-528B-4A3C-8950-BEECC189ADF7}">
+  <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="48" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.3828125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="46.84375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.69140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23.53515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="43.53515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="11.69140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="25.3046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.69140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -568,259 +554,76 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
       </c>
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
         <v>17</v>
       </c>
-      <c r="H4" t="s">
-        <v>15</v>
-      </c>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" t="s">
-        <v>15</v>
-      </c>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" t="s">
-        <v>15</v>
-      </c>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" t="s">
-        <v>20</v>
-      </c>
-      <c r="H7" t="s">
-        <v>15</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
-        <v>15</v>
-      </c>
-      <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="K3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H9" t="s">
-        <v>15</v>
-      </c>
-      <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" t="s">
-        <v>15</v>
-      </c>
-      <c r="K10" s="1"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0" pivotTables="0"/>

</xml_diff>